<commit_message>
corrección incisión y agregado de botón borrar evento
</commit_message>
<xml_diff>
--- a/Codigos/Raspberry/Registro Eventos.xlsx
+++ b/Codigos/Raspberry/Registro Eventos.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zakie Assad\Proyecto Final\Presentacion\Version Final Codigos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zakie Assad\Proyecto Final\Git\MoAna\Codigos\Raspberry\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF8E3574-15DE-42EA-8771-2879AA697C3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44CD11A5-DD19-49FF-8EA1-79B575AB9B97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3270" yWindow="0" windowWidth="15375" windowHeight="10800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -52,9 +52,6 @@
     <t>DICLOFENAC</t>
   </si>
   <si>
-    <t>INSICIÓN</t>
-  </si>
-  <si>
     <t>DIPIRONA</t>
   </si>
   <si>
@@ -92,6 +89,9 @@
   </si>
   <si>
     <t>TRAMADOL</t>
+  </si>
+  <si>
+    <t>INCISIÓN</t>
   </si>
 </sst>
 </file>
@@ -496,7 +496,7 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="C4" t="s">
         <v>8</v>
@@ -507,63 +507,63 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>